<commit_message>
Update: New faction-landmark + maptile/global explore button
</commit_message>
<xml_diff>
--- a/tts_envs/data/maptile.xlsx
+++ b/tts_envs/data/maptile.xlsx
@@ -14,10 +14,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="backs" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="biome_descriptions" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="maptile_table" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="exploration" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="density" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="weights" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tiers" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="explore_outcomes" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="exploration" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="density" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="weights" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tiers" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="landmark_table" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -6825,6 +6827,2134 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:P42"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="50" customWidth="1" min="16" max="16"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>biome</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>fishing</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>mining</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>forestry</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>hunting</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>herbalism</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>resource_none</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>camp</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>cave</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>caravan</t>
+        </is>
+      </c>
+      <c r="K1" s="4" t="inlineStr">
+        <is>
+          <t>beehive</t>
+        </is>
+      </c>
+      <c r="L1" s="4" t="inlineStr">
+        <is>
+          <t>shrine</t>
+        </is>
+      </c>
+      <c r="M1" s="4" t="inlineStr">
+        <is>
+          <t>warehouse</t>
+        </is>
+      </c>
+      <c r="N1" s="4" t="inlineStr">
+        <is>
+          <t>bank</t>
+        </is>
+      </c>
+      <c r="O1" s="4" t="inlineStr">
+        <is>
+          <t>poi_none</t>
+        </is>
+      </c>
+      <c r="P1" s="4" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>forest</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" t="n">
+        <v>6</v>
+      </c>
+      <c r="E2" t="n">
+        <v>4</v>
+      </c>
+      <c r="F2" t="n">
+        <v>4</v>
+      </c>
+      <c r="G2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" t="n">
+        <v>4</v>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>SAMPLE weights: relative odds within Resources (fishing..resource_none) and within Points of interest (camp..poi_none); 0 = never</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>plains</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>6</v>
+      </c>
+      <c r="F3" t="n">
+        <v>5</v>
+      </c>
+      <c r="G3" t="n">
+        <v>4</v>
+      </c>
+      <c r="H3" t="n">
+        <v>2</v>
+      </c>
+      <c r="I3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>town</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>city</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>2</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>mountain</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" t="n">
+        <v>8</v>
+      </c>
+      <c r="D6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" t="n">
+        <v>3</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" t="n">
+        <v>2</v>
+      </c>
+      <c r="H6" t="n">
+        <v>2</v>
+      </c>
+      <c r="I6" t="n">
+        <v>5</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>guildhall</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
+        <v>2</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>riverside</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" t="n">
+        <v>3</v>
+      </c>
+      <c r="F8" t="n">
+        <v>3</v>
+      </c>
+      <c r="G8" t="n">
+        <v>2</v>
+      </c>
+      <c r="H8" t="n">
+        <v>2</v>
+      </c>
+      <c r="I8" t="n">
+        <v>1</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>marsh</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>4</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
+        <v>3</v>
+      </c>
+      <c r="F9" t="n">
+        <v>6</v>
+      </c>
+      <c r="G9" t="n">
+        <v>2</v>
+      </c>
+      <c r="H9" t="n">
+        <v>2</v>
+      </c>
+      <c r="I9" t="n">
+        <v>1</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>hills</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" t="n">
+        <v>4</v>
+      </c>
+      <c r="D10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" t="n">
+        <v>5</v>
+      </c>
+      <c r="F10" t="n">
+        <v>3</v>
+      </c>
+      <c r="G10" t="n">
+        <v>2</v>
+      </c>
+      <c r="H10" t="n">
+        <v>2</v>
+      </c>
+      <c r="I10" t="n">
+        <v>5</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0</v>
+      </c>
+      <c r="N10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>blossomgrove</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" t="n">
+        <v>3</v>
+      </c>
+      <c r="E11" t="n">
+        <v>2</v>
+      </c>
+      <c r="F11" t="n">
+        <v>7</v>
+      </c>
+      <c r="G11" t="n">
+        <v>2</v>
+      </c>
+      <c r="H11" t="n">
+        <v>3</v>
+      </c>
+      <c r="I11" t="n">
+        <v>1</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>mushroomhollow</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" t="n">
+        <v>2</v>
+      </c>
+      <c r="E12" t="n">
+        <v>2</v>
+      </c>
+      <c r="F12" t="n">
+        <v>7</v>
+      </c>
+      <c r="G12" t="n">
+        <v>2</v>
+      </c>
+      <c r="H12" t="n">
+        <v>3</v>
+      </c>
+      <c r="I12" t="n">
+        <v>1</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>deepwood</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" t="n">
+        <v>6</v>
+      </c>
+      <c r="E13" t="n">
+        <v>5</v>
+      </c>
+      <c r="F13" t="n">
+        <v>3</v>
+      </c>
+      <c r="G13" t="n">
+        <v>2</v>
+      </c>
+      <c r="H13" t="n">
+        <v>3</v>
+      </c>
+      <c r="I13" t="n">
+        <v>1</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>heath</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" t="n">
+        <v>4</v>
+      </c>
+      <c r="F14" t="n">
+        <v>6</v>
+      </c>
+      <c r="G14" t="n">
+        <v>4</v>
+      </c>
+      <c r="H14" t="n">
+        <v>2</v>
+      </c>
+      <c r="I14" t="n">
+        <v>1</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O14" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>ashland</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" t="n">
+        <v>5</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" t="n">
+        <v>6</v>
+      </c>
+      <c r="H15" t="n">
+        <v>4</v>
+      </c>
+      <c r="I15" t="n">
+        <v>2</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>ruins</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" t="n">
+        <v>3</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" t="n">
+        <v>4</v>
+      </c>
+      <c r="H16" t="n">
+        <v>4</v>
+      </c>
+      <c r="I16" t="n">
+        <v>2</v>
+      </c>
+      <c r="J16" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>quarry</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" t="n">
+        <v>9</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" t="n">
+        <v>2</v>
+      </c>
+      <c r="H17" t="n">
+        <v>2</v>
+      </c>
+      <c r="I17" t="n">
+        <v>5</v>
+      </c>
+      <c r="J17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" t="n">
+        <v>0</v>
+      </c>
+      <c r="N17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O17" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>lumbercamp</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" t="n">
+        <v>9</v>
+      </c>
+      <c r="E18" t="n">
+        <v>2</v>
+      </c>
+      <c r="F18" t="n">
+        <v>1</v>
+      </c>
+      <c r="G18" t="n">
+        <v>2</v>
+      </c>
+      <c r="H18" t="n">
+        <v>3</v>
+      </c>
+      <c r="I18" t="n">
+        <v>1</v>
+      </c>
+      <c r="J18" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" t="n">
+        <v>0</v>
+      </c>
+      <c r="M18" t="n">
+        <v>0</v>
+      </c>
+      <c r="N18" t="n">
+        <v>0</v>
+      </c>
+      <c r="O18" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>farmstead</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" t="n">
+        <v>3</v>
+      </c>
+      <c r="F19" t="n">
+        <v>4</v>
+      </c>
+      <c r="G19" t="n">
+        <v>2</v>
+      </c>
+      <c r="H19" t="n">
+        <v>2</v>
+      </c>
+      <c r="I19" t="n">
+        <v>1</v>
+      </c>
+      <c r="J19" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" t="n">
+        <v>0</v>
+      </c>
+      <c r="M19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N19" t="n">
+        <v>0</v>
+      </c>
+      <c r="O19" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>orchard</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" t="n">
+        <v>4</v>
+      </c>
+      <c r="E20" t="n">
+        <v>2</v>
+      </c>
+      <c r="F20" t="n">
+        <v>6</v>
+      </c>
+      <c r="G20" t="n">
+        <v>2</v>
+      </c>
+      <c r="H20" t="n">
+        <v>3</v>
+      </c>
+      <c r="I20" t="n">
+        <v>1</v>
+      </c>
+      <c r="J20" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" t="n">
+        <v>0</v>
+      </c>
+      <c r="M20" t="n">
+        <v>0</v>
+      </c>
+      <c r="N20" t="n">
+        <v>0</v>
+      </c>
+      <c r="O20" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>settlement</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" t="n">
+        <v>1</v>
+      </c>
+      <c r="G21" t="n">
+        <v>2</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" t="n">
+        <v>0</v>
+      </c>
+      <c r="J21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M21" t="n">
+        <v>0</v>
+      </c>
+      <c r="N21" t="n">
+        <v>0</v>
+      </c>
+      <c r="O21" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>lakeshore</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>8</v>
+      </c>
+      <c r="C22" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F22" t="n">
+        <v>2</v>
+      </c>
+      <c r="G22" t="n">
+        <v>2</v>
+      </c>
+      <c r="H22" t="n">
+        <v>2</v>
+      </c>
+      <c r="I22" t="n">
+        <v>1</v>
+      </c>
+      <c r="J22" t="n">
+        <v>0</v>
+      </c>
+      <c r="K22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L22" t="n">
+        <v>0</v>
+      </c>
+      <c r="M22" t="n">
+        <v>0</v>
+      </c>
+      <c r="N22" t="n">
+        <v>0</v>
+      </c>
+      <c r="O22" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>briarthicket</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" t="n">
+        <v>3</v>
+      </c>
+      <c r="E23" t="n">
+        <v>5</v>
+      </c>
+      <c r="F23" t="n">
+        <v>5</v>
+      </c>
+      <c r="G23" t="n">
+        <v>4</v>
+      </c>
+      <c r="H23" t="n">
+        <v>3</v>
+      </c>
+      <c r="I23" t="n">
+        <v>1</v>
+      </c>
+      <c r="J23" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" t="n">
+        <v>0</v>
+      </c>
+      <c r="L23" t="n">
+        <v>0</v>
+      </c>
+      <c r="M23" t="n">
+        <v>0</v>
+      </c>
+      <c r="N23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O23" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>wildflowermeadow</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" t="n">
+        <v>3</v>
+      </c>
+      <c r="F24" t="n">
+        <v>9</v>
+      </c>
+      <c r="G24" t="n">
+        <v>2</v>
+      </c>
+      <c r="H24" t="n">
+        <v>2</v>
+      </c>
+      <c r="I24" t="n">
+        <v>1</v>
+      </c>
+      <c r="J24" t="n">
+        <v>0</v>
+      </c>
+      <c r="K24" t="n">
+        <v>0</v>
+      </c>
+      <c r="L24" t="n">
+        <v>0</v>
+      </c>
+      <c r="M24" t="n">
+        <v>0</v>
+      </c>
+      <c r="N24" t="n">
+        <v>0</v>
+      </c>
+      <c r="O24" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>canyon</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" t="n">
+        <v>6</v>
+      </c>
+      <c r="D25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F25" t="n">
+        <v>1</v>
+      </c>
+      <c r="G25" t="n">
+        <v>4</v>
+      </c>
+      <c r="H25" t="n">
+        <v>2</v>
+      </c>
+      <c r="I25" t="n">
+        <v>5</v>
+      </c>
+      <c r="J25" t="n">
+        <v>0</v>
+      </c>
+      <c r="K25" t="n">
+        <v>0</v>
+      </c>
+      <c r="L25" t="n">
+        <v>0</v>
+      </c>
+      <c r="M25" t="n">
+        <v>0</v>
+      </c>
+      <c r="N25" t="n">
+        <v>0</v>
+      </c>
+      <c r="O25" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>waterfallcliffs</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>6</v>
+      </c>
+      <c r="C26" t="n">
+        <v>3</v>
+      </c>
+      <c r="D26" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" t="n">
+        <v>1</v>
+      </c>
+      <c r="F26" t="n">
+        <v>2</v>
+      </c>
+      <c r="G26" t="n">
+        <v>2</v>
+      </c>
+      <c r="H26" t="n">
+        <v>2</v>
+      </c>
+      <c r="I26" t="n">
+        <v>5</v>
+      </c>
+      <c r="J26" t="n">
+        <v>0</v>
+      </c>
+      <c r="K26" t="n">
+        <v>0</v>
+      </c>
+      <c r="L26" t="n">
+        <v>0</v>
+      </c>
+      <c r="M26" t="n">
+        <v>0</v>
+      </c>
+      <c r="N26" t="n">
+        <v>0</v>
+      </c>
+      <c r="O26" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>standingstones</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" t="n">
+        <v>2</v>
+      </c>
+      <c r="D27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" t="n">
+        <v>1</v>
+      </c>
+      <c r="F27" t="n">
+        <v>3</v>
+      </c>
+      <c r="G27" t="n">
+        <v>2</v>
+      </c>
+      <c r="H27" t="n">
+        <v>2</v>
+      </c>
+      <c r="I27" t="n">
+        <v>5</v>
+      </c>
+      <c r="J27" t="n">
+        <v>0</v>
+      </c>
+      <c r="K27" t="n">
+        <v>0</v>
+      </c>
+      <c r="L27" t="n">
+        <v>0</v>
+      </c>
+      <c r="M27" t="n">
+        <v>0</v>
+      </c>
+      <c r="N27" t="n">
+        <v>0</v>
+      </c>
+      <c r="O27" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>battlefield</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" t="n">
+        <v>1</v>
+      </c>
+      <c r="D28" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" t="n">
+        <v>2</v>
+      </c>
+      <c r="F28" t="n">
+        <v>1</v>
+      </c>
+      <c r="G28" t="n">
+        <v>6</v>
+      </c>
+      <c r="H28" t="n">
+        <v>4</v>
+      </c>
+      <c r="I28" t="n">
+        <v>2</v>
+      </c>
+      <c r="J28" t="n">
+        <v>0</v>
+      </c>
+      <c r="K28" t="n">
+        <v>0</v>
+      </c>
+      <c r="L28" t="n">
+        <v>0</v>
+      </c>
+      <c r="M28" t="n">
+        <v>0</v>
+      </c>
+      <c r="N28" t="n">
+        <v>0</v>
+      </c>
+      <c r="O28" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>hotsprings</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>2</v>
+      </c>
+      <c r="C29" t="n">
+        <v>3</v>
+      </c>
+      <c r="D29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" t="n">
+        <v>1</v>
+      </c>
+      <c r="F29" t="n">
+        <v>5</v>
+      </c>
+      <c r="G29" t="n">
+        <v>2</v>
+      </c>
+      <c r="H29" t="n">
+        <v>2</v>
+      </c>
+      <c r="I29" t="n">
+        <v>1</v>
+      </c>
+      <c r="J29" t="n">
+        <v>0</v>
+      </c>
+      <c r="K29" t="n">
+        <v>0</v>
+      </c>
+      <c r="L29" t="n">
+        <v>0</v>
+      </c>
+      <c r="M29" t="n">
+        <v>0</v>
+      </c>
+      <c r="N29" t="n">
+        <v>0</v>
+      </c>
+      <c r="O29" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>lilypond</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>7</v>
+      </c>
+      <c r="C30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" t="n">
+        <v>2</v>
+      </c>
+      <c r="F30" t="n">
+        <v>5</v>
+      </c>
+      <c r="G30" t="n">
+        <v>2</v>
+      </c>
+      <c r="H30" t="n">
+        <v>2</v>
+      </c>
+      <c r="I30" t="n">
+        <v>1</v>
+      </c>
+      <c r="J30" t="n">
+        <v>0</v>
+      </c>
+      <c r="K30" t="n">
+        <v>0</v>
+      </c>
+      <c r="L30" t="n">
+        <v>0</v>
+      </c>
+      <c r="M30" t="n">
+        <v>0</v>
+      </c>
+      <c r="N30" t="n">
+        <v>0</v>
+      </c>
+      <c r="O30" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>otterwharf</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>8</v>
+      </c>
+      <c r="C31" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" t="n">
+        <v>2</v>
+      </c>
+      <c r="H31" t="n">
+        <v>2</v>
+      </c>
+      <c r="I31" t="n">
+        <v>1</v>
+      </c>
+      <c r="J31" t="n">
+        <v>0</v>
+      </c>
+      <c r="K31" t="n">
+        <v>0</v>
+      </c>
+      <c r="L31" t="n">
+        <v>0</v>
+      </c>
+      <c r="M31" t="n">
+        <v>0</v>
+      </c>
+      <c r="N31" t="n">
+        <v>0</v>
+      </c>
+      <c r="O31" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>drownedwood</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>4</v>
+      </c>
+      <c r="C32" t="n">
+        <v>0</v>
+      </c>
+      <c r="D32" t="n">
+        <v>4</v>
+      </c>
+      <c r="E32" t="n">
+        <v>2</v>
+      </c>
+      <c r="F32" t="n">
+        <v>3</v>
+      </c>
+      <c r="G32" t="n">
+        <v>2</v>
+      </c>
+      <c r="H32" t="n">
+        <v>2</v>
+      </c>
+      <c r="I32" t="n">
+        <v>1</v>
+      </c>
+      <c r="J32" t="n">
+        <v>0</v>
+      </c>
+      <c r="K32" t="n">
+        <v>0</v>
+      </c>
+      <c r="L32" t="n">
+        <v>0</v>
+      </c>
+      <c r="M32" t="n">
+        <v>0</v>
+      </c>
+      <c r="N32" t="n">
+        <v>0</v>
+      </c>
+      <c r="O32" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>watermill</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>5</v>
+      </c>
+      <c r="C33" t="n">
+        <v>0</v>
+      </c>
+      <c r="D33" t="n">
+        <v>1</v>
+      </c>
+      <c r="E33" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" t="n">
+        <v>2</v>
+      </c>
+      <c r="G33" t="n">
+        <v>2</v>
+      </c>
+      <c r="H33" t="n">
+        <v>2</v>
+      </c>
+      <c r="I33" t="n">
+        <v>1</v>
+      </c>
+      <c r="J33" t="n">
+        <v>0</v>
+      </c>
+      <c r="K33" t="n">
+        <v>0</v>
+      </c>
+      <c r="L33" t="n">
+        <v>0</v>
+      </c>
+      <c r="M33" t="n">
+        <v>0</v>
+      </c>
+      <c r="N33" t="n">
+        <v>0</v>
+      </c>
+      <c r="O33" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>beaverdam</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>5</v>
+      </c>
+      <c r="C34" t="n">
+        <v>0</v>
+      </c>
+      <c r="D34" t="n">
+        <v>6</v>
+      </c>
+      <c r="E34" t="n">
+        <v>2</v>
+      </c>
+      <c r="F34" t="n">
+        <v>1</v>
+      </c>
+      <c r="G34" t="n">
+        <v>2</v>
+      </c>
+      <c r="H34" t="n">
+        <v>2</v>
+      </c>
+      <c r="I34" t="n">
+        <v>1</v>
+      </c>
+      <c r="J34" t="n">
+        <v>0</v>
+      </c>
+      <c r="K34" t="n">
+        <v>0</v>
+      </c>
+      <c r="L34" t="n">
+        <v>0</v>
+      </c>
+      <c r="M34" t="n">
+        <v>0</v>
+      </c>
+      <c r="N34" t="n">
+        <v>0</v>
+      </c>
+      <c r="O34" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>barrows</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" t="n">
+        <v>2</v>
+      </c>
+      <c r="D35" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" t="n">
+        <v>2</v>
+      </c>
+      <c r="G35" t="n">
+        <v>4</v>
+      </c>
+      <c r="H35" t="n">
+        <v>4</v>
+      </c>
+      <c r="I35" t="n">
+        <v>4</v>
+      </c>
+      <c r="J35" t="n">
+        <v>0</v>
+      </c>
+      <c r="K35" t="n">
+        <v>0</v>
+      </c>
+      <c r="L35" t="n">
+        <v>0</v>
+      </c>
+      <c r="M35" t="n">
+        <v>0</v>
+      </c>
+      <c r="N35" t="n">
+        <v>0</v>
+      </c>
+      <c r="O35" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>slagworks</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" t="n">
+        <v>8</v>
+      </c>
+      <c r="D36" t="n">
+        <v>0</v>
+      </c>
+      <c r="E36" t="n">
+        <v>0</v>
+      </c>
+      <c r="F36" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" t="n">
+        <v>4</v>
+      </c>
+      <c r="H36" t="n">
+        <v>4</v>
+      </c>
+      <c r="I36" t="n">
+        <v>2</v>
+      </c>
+      <c r="J36" t="n">
+        <v>0</v>
+      </c>
+      <c r="K36" t="n">
+        <v>0</v>
+      </c>
+      <c r="L36" t="n">
+        <v>0</v>
+      </c>
+      <c r="M36" t="n">
+        <v>0</v>
+      </c>
+      <c r="N36" t="n">
+        <v>0</v>
+      </c>
+      <c r="O36" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>blightwood</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" t="n">
+        <v>0</v>
+      </c>
+      <c r="D37" t="n">
+        <v>4</v>
+      </c>
+      <c r="E37" t="n">
+        <v>3</v>
+      </c>
+      <c r="F37" t="n">
+        <v>4</v>
+      </c>
+      <c r="G37" t="n">
+        <v>4</v>
+      </c>
+      <c r="H37" t="n">
+        <v>3</v>
+      </c>
+      <c r="I37" t="n">
+        <v>1</v>
+      </c>
+      <c r="J37" t="n">
+        <v>0</v>
+      </c>
+      <c r="K37" t="n">
+        <v>0</v>
+      </c>
+      <c r="L37" t="n">
+        <v>0</v>
+      </c>
+      <c r="M37" t="n">
+        <v>0</v>
+      </c>
+      <c r="N37" t="n">
+        <v>0</v>
+      </c>
+      <c r="O37" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>cliffside</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" t="n">
+        <v>6</v>
+      </c>
+      <c r="D38" t="n">
+        <v>0</v>
+      </c>
+      <c r="E38" t="n">
+        <v>4</v>
+      </c>
+      <c r="F38" t="n">
+        <v>2</v>
+      </c>
+      <c r="G38" t="n">
+        <v>2</v>
+      </c>
+      <c r="H38" t="n">
+        <v>2</v>
+      </c>
+      <c r="I38" t="n">
+        <v>5</v>
+      </c>
+      <c r="J38" t="n">
+        <v>0</v>
+      </c>
+      <c r="K38" t="n">
+        <v>0</v>
+      </c>
+      <c r="L38" t="n">
+        <v>0</v>
+      </c>
+      <c r="M38" t="n">
+        <v>0</v>
+      </c>
+      <c r="N38" t="n">
+        <v>0</v>
+      </c>
+      <c r="O38" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>coldmountain</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" t="n">
+        <v>7</v>
+      </c>
+      <c r="D39" t="n">
+        <v>1</v>
+      </c>
+      <c r="E39" t="n">
+        <v>4</v>
+      </c>
+      <c r="F39" t="n">
+        <v>1</v>
+      </c>
+      <c r="G39" t="n">
+        <v>4</v>
+      </c>
+      <c r="H39" t="n">
+        <v>2</v>
+      </c>
+      <c r="I39" t="n">
+        <v>5</v>
+      </c>
+      <c r="J39" t="n">
+        <v>0</v>
+      </c>
+      <c r="K39" t="n">
+        <v>0</v>
+      </c>
+      <c r="L39" t="n">
+        <v>0</v>
+      </c>
+      <c r="M39" t="n">
+        <v>0</v>
+      </c>
+      <c r="N39" t="n">
+        <v>0</v>
+      </c>
+      <c r="O39" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>hillcentral</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" t="n">
+        <v>4</v>
+      </c>
+      <c r="D40" t="n">
+        <v>1</v>
+      </c>
+      <c r="E40" t="n">
+        <v>4</v>
+      </c>
+      <c r="F40" t="n">
+        <v>3</v>
+      </c>
+      <c r="G40" t="n">
+        <v>2</v>
+      </c>
+      <c r="H40" t="n">
+        <v>2</v>
+      </c>
+      <c r="I40" t="n">
+        <v>5</v>
+      </c>
+      <c r="J40" t="n">
+        <v>0</v>
+      </c>
+      <c r="K40" t="n">
+        <v>0</v>
+      </c>
+      <c r="L40" t="n">
+        <v>0</v>
+      </c>
+      <c r="M40" t="n">
+        <v>0</v>
+      </c>
+      <c r="N40" t="n">
+        <v>0</v>
+      </c>
+      <c r="O40" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>battlefieldmountain</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" t="n">
+        <v>4</v>
+      </c>
+      <c r="D41" t="n">
+        <v>0</v>
+      </c>
+      <c r="E41" t="n">
+        <v>2</v>
+      </c>
+      <c r="F41" t="n">
+        <v>1</v>
+      </c>
+      <c r="G41" t="n">
+        <v>6</v>
+      </c>
+      <c r="H41" t="n">
+        <v>2</v>
+      </c>
+      <c r="I41" t="n">
+        <v>5</v>
+      </c>
+      <c r="J41" t="n">
+        <v>0</v>
+      </c>
+      <c r="K41" t="n">
+        <v>0</v>
+      </c>
+      <c r="L41" t="n">
+        <v>0</v>
+      </c>
+      <c r="M41" t="n">
+        <v>0</v>
+      </c>
+      <c r="N41" t="n">
+        <v>0</v>
+      </c>
+      <c r="O41" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>battlefieldwaterside</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>4</v>
+      </c>
+      <c r="C42" t="n">
+        <v>0</v>
+      </c>
+      <c r="D42" t="n">
+        <v>0</v>
+      </c>
+      <c r="E42" t="n">
+        <v>2</v>
+      </c>
+      <c r="F42" t="n">
+        <v>1</v>
+      </c>
+      <c r="G42" t="n">
+        <v>6</v>
+      </c>
+      <c r="H42" t="n">
+        <v>4</v>
+      </c>
+      <c r="I42" t="n">
+        <v>2</v>
+      </c>
+      <c r="J42" t="n">
+        <v>0</v>
+      </c>
+      <c r="K42" t="n">
+        <v>0</v>
+      </c>
+      <c r="L42" t="n">
+        <v>0</v>
+      </c>
+      <c r="M42" t="n">
+        <v>0</v>
+      </c>
+      <c r="N42" t="n">
+        <v>0</v>
+      </c>
+      <c r="O42" t="n">
+        <v>4</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -6894,7 +9024,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7152,7 +9282,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7257,6 +9387,42 @@
       <c r="D4" t="inlineStr">
         <is>
           <t>city</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>gmnotes</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>actions</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>notes</t>
         </is>
       </c>
     </row>
@@ -66989,7 +69155,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J42"/>
+  <dimension ref="A1:T42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="6"/>
@@ -67002,6 +69168,16 @@
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="50" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="19" max="19"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="1" s="2">
@@ -67053,6 +69229,56 @@
       <c r="J1" s="4" t="inlineStr">
         <is>
           <t>notes</t>
+        </is>
+      </c>
+      <c r="K1" s="4" t="inlineStr">
+        <is>
+          <t>spawnmeeple1_gmnotes</t>
+        </is>
+      </c>
+      <c r="L1" s="4" t="inlineStr">
+        <is>
+          <t>spawnmeeple1_memo</t>
+        </is>
+      </c>
+      <c r="M1" s="4" t="inlineStr">
+        <is>
+          <t>spawnmeeple2_gmnotes</t>
+        </is>
+      </c>
+      <c r="N1" s="4" t="inlineStr">
+        <is>
+          <t>spawnmeeple2_memo</t>
+        </is>
+      </c>
+      <c r="O1" s="4" t="inlineStr">
+        <is>
+          <t>spawnlandmark1_gmnotes</t>
+        </is>
+      </c>
+      <c r="P1" s="4" t="inlineStr">
+        <is>
+          <t>spawnlandmark1_memo</t>
+        </is>
+      </c>
+      <c r="Q1" s="4" t="inlineStr">
+        <is>
+          <t>spawnlandmark2_gmnotes</t>
+        </is>
+      </c>
+      <c r="R1" s="4" t="inlineStr">
+        <is>
+          <t>spawnlandmark2_memo</t>
+        </is>
+      </c>
+      <c r="S1" s="4" t="inlineStr">
+        <is>
+          <t>spawnlandmark3_gmnotes</t>
+        </is>
+      </c>
+      <c r="T1" s="4" t="inlineStr">
+        <is>
+          <t>spawnlandmark3_memo</t>
         </is>
       </c>
     </row>
@@ -67354,50 +69580,62 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G42"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="6"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="50" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="90" customWidth="1" min="8" max="8"/>
+    <col width="50" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="1" s="2">
+    <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>biome</t>
+          <t>outcome</t>
         </is>
       </c>
       <c r="B1" s="4" t="inlineStr">
         <is>
-          <t>spawn1</t>
+          <t>category</t>
         </is>
       </c>
       <c r="C1" s="4" t="inlineStr">
         <is>
-          <t>spawn2</t>
+          <t>kind</t>
         </is>
       </c>
       <c r="D1" s="4" t="inlineStr">
         <is>
-          <t>spawn3</t>
+          <t>name</t>
         </is>
       </c>
       <c r="E1" s="4" t="inlineStr">
         <is>
-          <t>spawnmeeple1</t>
+          <t>landmarks</t>
         </is>
       </c>
       <c r="F1" s="4" t="inlineStr">
         <is>
-          <t>spawngold</t>
+          <t>gmnotes</t>
         </is>
       </c>
       <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>memo</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>flavor</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
@@ -67406,292 +69644,500 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>forest</t>
+          <t>fishing</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>resource</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>landmark</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Fishing</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Fishing Node</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>DRAFT, not read by any sync yet -- see plans/auto_TODO.md 'Explore action'</t>
+          <t>biome={biome}</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>A slow, deep pool under the bank, and fish rising where nobody has cast a line in weeks.|Someone left a cracked rod wedged in the reeds. The fish here have clearly been winning.</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>gmnotes blank = keep the landmark's own kind (tokens.xlsx landmarks gmnotes; Global keys its buttons on it). memo {biome} = the tile's biome</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>plains</t>
+          <t>mining</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>resource</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>landmark</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Mining</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Mineral Node</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>biome={biome}</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>The ground has split along an old seam, and the rock inside glints when you scrape it.|Pick marks on the stone, years old. Whoever started this seam left in a hurry, and left the best of it.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>city</t>
+          <t>forestry</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>resource</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>landmark</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Forestry</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Forestry Node</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>biome={biome}</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>A stand of straight, seasoned timber. Someone notched the nearest trunk and never came back to finish.|Wind has brought down a sound old trunk across the path, already dry enough to work.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>mountain</t>
+          <t>hunting</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>resource</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>landmark</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Hunting</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Hunting Node</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>biome={biome}</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Fresh tracks, deep and close together, heading somewhere they have clearly been before.|A worn run through the grass, a tuft of fur on a thorn, and droppings still warm.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>guildhall</t>
+          <t>herbalism</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>resource</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>landmark</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Herbalism</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Herb Node</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>biome={biome}</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Bitterleaf grows thick where the ground stays damp, untouched by anything but bees.|Feverfew and sorrel crowd a sunny hollow. Someone has picked here before, carefully, leaving the roots.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>riverside</t>
+          <t>resource_none</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>resource</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>nothing</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Nothing</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>You search until your paws ache and find only stones that are just stones.|You turn over half the ground and find nothing worth the weight of carrying it.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>marsh</t>
+          <t>camp</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>poi</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>landmark</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Bandit camp</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Knave Camp|Knave Camp|Knave Encampment</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Smoke from a cookfire and a ring of tents nobody bothered to hide. Whoever camps here expects no trouble.|A knave camp: stolen pots, a lookout asleep on a crate, and more bedrolls than you would like.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>hills</t>
+          <t>cave</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>poi</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>landmark</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Cave</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Hollow|Hollow|Hollow|Burrow|Burrow|Cave|Warren</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>A cold breath comes out of a hole in the earth. Something has been dragging things inside.|Steps cut into the earth lead down into the dark. The bottom ones are worn smoother than the top.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>blossomgrove</t>
+          <t>caravan</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>poi</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>landmark</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Caravan</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>A string of painted wagons has stopped to rest the beasts. The drivers are going your way, for a price.</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>no landmark art yet: keep weight 0</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>mushroomhollow</t>
+          <t>beehive</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>poi</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>landmark</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Beehive</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>You hear the hive before you see it: a hollow trunk heavy with comb, and very busy.</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>no landmark art yet: keep weight 0</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>deepwood</t>
+          <t>shrine</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>poi</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>landmark</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Shrine</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>A little stone shrine, moss on its roof and fresh berries on its step. Someone still keeps it.</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>no landmark art yet: keep weight 0</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>heath</t>
+          <t>warehouse</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>poi</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>landmark</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Warehouse</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>A locked storehouse with a sound roof and a sign nailed to the door: GOODS KEPT. ASK NO ONE.</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>no landmark art yet: keep weight 0</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ashland</t>
+          <t>bank</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>poi</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>landmark</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Bank</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>A squat strongroom with three locks, every one of them newer than the walls.</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>no landmark art yet: keep weight 0</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ruins</t>
+          <t>poi_none</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>poi</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>nothing</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Nothing</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>You walk the edges of the place and find nothing worth putting on a map.|A promising shape in the distance turns out to be a stump.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>quarry</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>lumbercamp</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>farmstead</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>orchard</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>lakeshore</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>briarthicket</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>wildflowermeadow</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>canyon</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>waterfallcliffs</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>standingstones</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>battlefield</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>hotsprings</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>settlement</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>town</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>lilypond</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>otterwharf</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>drownedwood</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>watermill</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>beaverdam</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>barrows</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>slagworks</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>blightwood</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>cliffside</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>coldmountain</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>hillcentral</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>battlefieldmountain</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>battlefieldwaterside</t>
+          <t>event</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>event</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>nothing</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Experience</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>You leave the path to find whoever lives here, and somebody finds you first.|You go knocking on whatever passes for doors around here.</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Experiences: flavor only, draws the region's top event card</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update: faction capitol landmark resize
</commit_message>
<xml_diff>
--- a/tts_envs/data/maptile.xlsx
+++ b/tts_envs/data/maptile.xlsx
@@ -16,10 +16,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="maptile_table" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="explore_outcomes" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="exploration" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="density" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="weights" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tiers" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="landmark_table" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="explore_special" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="density" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="weights" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tiers" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="landmark_table" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -8955,6 +8956,81 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="90" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>biome</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>label</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>tooltip</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>flavor</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>guildhall</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Eat</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Share a meal at the guildhall. Uses up an explore.</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>The guild cook ladles out stew and asks no questions about where you have been.|Bread, cheese and a pot of tea that has been kept warm since morning, just in case.</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>spends an explore; effect is announced only for now (Game design 'Time, food, hunger')</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -9024,7 +9100,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -9282,7 +9358,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -9395,7 +9471,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>